<commit_message>
data: updated BU mapping + rebuild aggregations v10
Bajaj Mapping.xlsx: +7 new models (MC+2, CV+3, UB+2)
  MC: Pulsar N150, Pulsar 180
  CV: WEGO P9018, WEGO P70, WEGO C90
  UB: Chetak 2903, Chetak C2501

All 39k previously unmatched Bajaj leads now properly classified:
  MC: 664k→670k  |  UB: 154k→188k  |  CV: 111k (stable)
  "Bajaj" fallback bucket: eliminated (was 39k)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Bajaj Mapping.xlsx
+++ b/Bajaj Mapping.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adityakumar/Downloads/Ather/Ather 2/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adityakumar/Downloads/Bajaj/cps-lead-dashboard/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F20A56DB-B9AB-2946-8D17-68ABD51A177C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCC2B0FC-498B-B54D-8136-2691B51F1AB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="16180" xr2:uid="{9042D7FF-378F-0C4B-A817-B24004E25046}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="71">
   <si>
     <t>Bajaj</t>
   </si>
@@ -231,6 +231,27 @@
   </si>
   <si>
     <t>Model Name</t>
+  </si>
+  <si>
+    <t>Bajaj Chetak 2903</t>
+  </si>
+  <si>
+    <t>Bajaj Chetak C2501</t>
+  </si>
+  <si>
+    <t>Bajaj Pulsar N150</t>
+  </si>
+  <si>
+    <t>Bajaj Pulsar 180</t>
+  </si>
+  <si>
+    <t>Bajaj WEGO P9018</t>
+  </si>
+  <si>
+    <t>Bajaj WEGO P70</t>
+  </si>
+  <si>
+    <t>Bajaj WEGO C90</t>
   </si>
 </sst>
 </file>
@@ -642,7 +663,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6A6C1A8-F9DF-DF4E-9D31-E1A661CB5774}">
-  <dimension ref="A1:C55"/>
+  <dimension ref="A1:C62"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14.33203125" bestFit="1" customWidth="1"/>
@@ -1255,6 +1276,83 @@
         <v>61</v>
       </c>
     </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A56" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B56" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C56" s="2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A57" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B57" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C57" s="2" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A58" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B58" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C58" s="2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A59" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B59" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C59" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A60" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C60" s="2" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A61" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B61" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C61" s="2" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A62" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B62" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C62" s="2" t="s">
+        <v>70</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Update Bajaj Mapping.xlsx: add Jawa/Yezdi/BSA model→BU mappings
Adds 12 new entries for Jawa brand models mapping to BUs:
Jawa (Jawa 42, Jawa 42 Bobber, Jawa Perak),
Yezdi (Jawa 350, Yezdi Scrambler, Yezdi Roadster, Yezdi Adventure, Yezdi Scrambler 350),
BSA (Jawa 42 FJ, BSA Scrambler 650, BSA Gold Star)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Bajaj Mapping.xlsx
+++ b/Bajaj Mapping.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10517"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10525"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adityakumar/Downloads/Bajaj/cps-lead-dashboard/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCC2B0FC-498B-B54D-8136-2691B51F1AB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA5DE7CC-8999-5944-9A8E-08F46CA3D2A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="16180" xr2:uid="{9042D7FF-378F-0C4B-A817-B24004E25046}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="86">
   <si>
     <t>Bajaj</t>
   </si>
@@ -252,6 +252,51 @@
   </si>
   <si>
     <t>Bajaj WEGO C90</t>
+  </si>
+  <si>
+    <t>Jawa</t>
+  </si>
+  <si>
+    <t>Jawa 42 Bobber</t>
+  </si>
+  <si>
+    <t>Yezdi</t>
+  </si>
+  <si>
+    <t>Jawa 350</t>
+  </si>
+  <si>
+    <t>BSA</t>
+  </si>
+  <si>
+    <t>Jawa 42 FJ</t>
+  </si>
+  <si>
+    <t>Yezdi Scrambler</t>
+  </si>
+  <si>
+    <t>Jawa 42</t>
+  </si>
+  <si>
+    <t>Jawa Perak</t>
+  </si>
+  <si>
+    <t>Yezdi Roadster</t>
+  </si>
+  <si>
+    <t>Yezdi Adventure</t>
+  </si>
+  <si>
+    <t>Yezdi Scrambler 350</t>
+  </si>
+  <si>
+    <t>BSA Scrambler 650</t>
+  </si>
+  <si>
+    <t>BSA Gold Star</t>
+  </si>
+  <si>
+    <t>2024 Yezdi Adventure</t>
   </si>
 </sst>
 </file>
@@ -663,7 +708,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6A6C1A8-F9DF-DF4E-9D31-E1A661CB5774}">
-  <dimension ref="A1:C62"/>
+  <dimension ref="A1:C74"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14.33203125" bestFit="1" customWidth="1"/>
@@ -1353,6 +1398,138 @@
         <v>70</v>
       </c>
     </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A63" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B63" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C63" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A64" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B64" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C64" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A65" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B65" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C65" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A66" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B66" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C66" s="2" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A67" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B67" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C67" s="2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A68" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B68" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C68" s="2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A69" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B69" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C69" s="2" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A70" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B70" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C70" s="2" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A71" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B71" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C71" s="2" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A72" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B72" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C72" s="2" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A73" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B73" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C73" s="2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A74" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B74" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C74" s="2" t="s">
+        <v>85</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>